<commit_message>
Sync Tencent documents and validate Luban configuration
Refresh 11 workbooks and 11 system documents from the master index. Fix missing Item metadata and reserved intelligence field names at the web source, then re-export. Add table and enum registration, generation script, source hashes, and evidence of strict generation and binary loading for all 14 tables.
</commit_message>
<xml_diff>
--- a/Excel/Character.xlsx
+++ b/Excel/Character.xlsx
@@ -17,12 +17,12 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>tc={767A0729-706D-48E8-84C5-1BACCCDE1903}</author>
-    <author>tc={D89F414D-F534-41E2-AF61-B8BCD9436A25}</author>
-    <author>tc={58A58356-4138-4117-8987-87074EDB5A3F}</author>
-    <author>tc={57C02C88-69AC-461B-AFD8-B043C6A9D729}</author>
-    <author>tc={A52EC4E5-B27B-4721-8A2F-83C56A5DF3E4}</author>
-    <author>tc={868567D7-992B-463D-8F0D-DE51E81A6259}</author>
+    <author>tc={83649CF8-8B92-455C-8E57-E1E0A90D1424}</author>
+    <author>tc={C4B0132B-5390-4AB2-B510-C2FC9166C06D}</author>
+    <author>tc={D6432E1B-FDE6-4CAD-86FC-5344C3986DFB}</author>
+    <author>tc={EAF807EC-876E-4906-A728-30425A8FAEB8}</author>
+    <author>tc={882642DE-C831-48D3-B6BD-88FEC39836B5}</author>
+    <author>tc={DADB90D3-59A9-45B0-9739-0C9B66E9E67E}</author>
   </authors>
   <commentList>
     <comment ref="E1" authorId="0">
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
   <si>
     <t/>
   </si>
@@ -314,6 +314,9 @@
   </si>
   <si>
     <t>trigger</t>
+  </si>
+  <si>
+    <t>intelligence</t>
   </si>
   <si>
     <r>
@@ -746,7 +749,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <tc2018:personList xmlns:tc2018="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="tc2018">
-  <tc2018:person displayName="空羽灵" id="{71050856-83C4-4C62-A593-2452975D3D98}"/>
+  <tc2018:person displayName="空羽灵" id="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}"/>
 </tc2018:personList>
 </file>
 
@@ -1013,7 +1016,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="">
-  <threadedComment ref="E1" dT="2026-10-08T14:09:11Z" personId="{71050856-83C4-4C62-A593-2452975D3D98}" id="{767A0729-706D-48E8-84C5-1BACCCDE1903}">
+  <threadedComment ref="E1" dT="2026-10-08T14:09:11Z" personId="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}" id="{83649CF8-8B92-455C-8E57-E1E0A90D1424}">
     <text>0=无
 1=厨师
 2=商人
@@ -1023,29 +1026,29 @@
 6=牧师
 7=吟游诗人</text>
   </threadedComment>
-  <threadedComment ref="D1" dT="2026-10-08T14:08:30Z" personId="{71050856-83C4-4C62-A593-2452975D3D98}" id="{D89F414D-F534-41E2-AF61-B8BCD9436A25}">
+  <threadedComment ref="D1" dT="2026-10-08T14:08:30Z" personId="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}" id="{C4B0132B-5390-4AB2-B510-C2FC9166C06D}">
     <text>1=男
 2=女</text>
   </threadedComment>
-  <threadedComment ref="Q1" dT="2026-10-08T14:10:50Z" personId="{71050856-83C4-4C62-A593-2452975D3D98}" id="{58A58356-4138-4117-8987-87074EDB5A3F}">
+  <threadedComment ref="Q1" dT="2026-10-08T14:10:50Z" personId="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}" id="{D6432E1B-FDE6-4CAD-86FC-5344C3986DFB}">
     <text>1=正常
 2=受伤
 3=中毒
 4=昏迷</text>
   </threadedComment>
-  <threadedComment ref="F1" dT="2026-10-08T14:09:40Z" personId="{71050856-83C4-4C62-A593-2452975D3D98}" id="{57C02C88-69AC-461B-AFD8-B043C6A9D729}">
+  <threadedComment ref="F1" dT="2026-10-08T14:09:40Z" personId="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}" id="{EAF807EC-876E-4906-A728-30425A8FAEB8}">
     <text>1=开朗
 2=沉稳
 3=谨慎</text>
   </threadedComment>
-  <threadedComment ref="G1" dT="2026-10-08T14:10:05Z" personId="{71050856-83C4-4C62-A593-2452975D3D98}" id="{A52EC4E5-B27B-4721-8A2F-83C56A5DF3E4}">
+  <threadedComment ref="G1" dT="2026-10-08T14:10:05Z" personId="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}" id="{882642DE-C831-48D3-B6BD-88FEC39836B5}">
     <text>1=烹饪
 2=锻造
 3=交易
 4=采集
 5=医术</text>
   </threadedComment>
-  <threadedComment ref="P1" dT="2026-10-08T14:10:27Z" personId="{71050856-83C4-4C62-A593-2452975D3D98}" id="{868567D7-992B-463D-8F0D-DE51E81A6259}">
+  <threadedComment ref="P1" dT="2026-10-08T14:10:27Z" personId="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}" id="{DADB90D3-59A9-45B0-9739-0C9B66E9E67E}">
     <text>1=平静
 2=愉快
 3=低落
@@ -1186,7 +1189,7 @@
         <v>35</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>36</v>
+        <v>74</v>
       </c>
       <c r="N2" s="7" t="s">
         <v>37</v>
@@ -8965,22 +8968,22 @@
         <v>1</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D1" s="20" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E1" s="20" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F1" s="20" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G1" s="20" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="24" customHeight="1">

</xml_diff>

<commit_message>
Update map locations and sync latest Tencent spreadsheets
</commit_message>
<xml_diff>
--- a/Excel/Character.xlsx
+++ b/Excel/Character.xlsx
@@ -17,12 +17,12 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>tc={83649CF8-8B92-455C-8E57-E1E0A90D1424}</author>
-    <author>tc={C4B0132B-5390-4AB2-B510-C2FC9166C06D}</author>
-    <author>tc={D6432E1B-FDE6-4CAD-86FC-5344C3986DFB}</author>
-    <author>tc={EAF807EC-876E-4906-A728-30425A8FAEB8}</author>
-    <author>tc={882642DE-C831-48D3-B6BD-88FEC39836B5}</author>
-    <author>tc={DADB90D3-59A9-45B0-9739-0C9B66E9E67E}</author>
+    <author>tc={FD08BDE2-6860-4554-85F0-37C9557D8847}</author>
+    <author>tc={6AF71D39-9D17-4F76-BBA8-3E2BDA78960F}</author>
+    <author>tc={616F167E-51F2-446C-978C-FCDCFF1D726C}</author>
+    <author>tc={0BFA0AE2-4038-4DAA-8BF8-1C45B4D2922A}</author>
+    <author>tc={02ECE897-F5AD-4A38-9D26-F436A9B034E3}</author>
+    <author>tc={54BF331E-D745-4386-A204-30D70EAD6E77}</author>
   </authors>
   <commentList>
     <comment ref="E1" authorId="0">
@@ -749,7 +749,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <tc2018:personList xmlns:tc2018="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="tc2018">
-  <tc2018:person displayName="空羽灵" id="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}"/>
+  <tc2018:person displayName="空羽灵" id="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}"/>
 </tc2018:personList>
 </file>
 
@@ -1016,7 +1016,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="">
-  <threadedComment ref="E1" dT="2026-10-08T14:09:11Z" personId="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}" id="{83649CF8-8B92-455C-8E57-E1E0A90D1424}">
+  <threadedComment ref="E1" dT="2026-10-08T14:09:11Z" personId="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}" id="{FD08BDE2-6860-4554-85F0-37C9557D8847}">
     <text>0=无
 1=厨师
 2=商人
@@ -1026,29 +1026,29 @@
 6=牧师
 7=吟游诗人</text>
   </threadedComment>
-  <threadedComment ref="D1" dT="2026-10-08T14:08:30Z" personId="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}" id="{C4B0132B-5390-4AB2-B510-C2FC9166C06D}">
+  <threadedComment ref="D1" dT="2026-10-08T14:08:30Z" personId="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}" id="{6AF71D39-9D17-4F76-BBA8-3E2BDA78960F}">
     <text>1=男
 2=女</text>
   </threadedComment>
-  <threadedComment ref="Q1" dT="2026-10-08T14:10:50Z" personId="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}" id="{D6432E1B-FDE6-4CAD-86FC-5344C3986DFB}">
+  <threadedComment ref="Q1" dT="2026-10-08T14:10:50Z" personId="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}" id="{616F167E-51F2-446C-978C-FCDCFF1D726C}">
     <text>1=正常
 2=受伤
 3=中毒
 4=昏迷</text>
   </threadedComment>
-  <threadedComment ref="F1" dT="2026-10-08T14:09:40Z" personId="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}" id="{EAF807EC-876E-4906-A728-30425A8FAEB8}">
+  <threadedComment ref="F1" dT="2026-10-08T14:09:40Z" personId="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}" id="{0BFA0AE2-4038-4DAA-8BF8-1C45B4D2922A}">
     <text>1=开朗
 2=沉稳
 3=谨慎</text>
   </threadedComment>
-  <threadedComment ref="G1" dT="2026-10-08T14:10:05Z" personId="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}" id="{882642DE-C831-48D3-B6BD-88FEC39836B5}">
+  <threadedComment ref="G1" dT="2026-10-08T14:10:05Z" personId="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}" id="{02ECE897-F5AD-4A38-9D26-F436A9B034E3}">
     <text>1=烹饪
 2=锻造
 3=交易
 4=采集
 5=医术</text>
   </threadedComment>
-  <threadedComment ref="P1" dT="2026-10-08T14:10:27Z" personId="{22F9DCCA-0D1D-4BD8-AB79-FC45ED83E33D}" id="{DADB90D3-59A9-45B0-9739-0C9B66E9E67E}">
+  <threadedComment ref="P1" dT="2026-10-08T14:10:27Z" personId="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}" id="{54BF331E-D745-4386-A204-30D70EAD6E77}">
     <text>1=平静
 2=愉快
 3=低落
@@ -1332,7 +1332,7 @@
         <v>3</v>
       </c>
       <c r="N4" s="14">
-        <f>=20+L4*5</f>
+        <f>20+L4*5</f>
         <v>30</v>
       </c>
       <c r="O4" s="10">
@@ -1400,7 +1400,7 @@
         <v>4</v>
       </c>
       <c r="N5" s="14">
-        <f>=20+L5*5</f>
+        <f>20+L5*5</f>
         <v>35</v>
       </c>
       <c r="O5" s="16">
@@ -1468,7 +1468,7 @@
         <v>2</v>
       </c>
       <c r="N6" s="14">
-        <f>=20+L6*5</f>
+        <f>20+L6*5</f>
         <v>45</v>
       </c>
       <c r="O6" s="16">
@@ -1536,7 +1536,7 @@
         <v>2</v>
       </c>
       <c r="N7" s="14">
-        <f>=20+L7*5</f>
+        <f>20+L7*5</f>
         <v>40</v>
       </c>
       <c r="O7" s="16">
@@ -1604,7 +1604,7 @@
         <v>5</v>
       </c>
       <c r="N8" s="14">
-        <f>=20+L8*5</f>
+        <f>20+L8*5</f>
         <v>25</v>
       </c>
       <c r="O8" s="16">
@@ -1648,7 +1648,7 @@
       <c r="L9" s="14" t="s"/>
       <c r="M9" s="14" t="s"/>
       <c r="N9" s="14" t="str">
-        <f>=IF(L9="","",20+L9*5)</f>
+        <f>IF(L9="","",20+L9*5)</f>
         <v/>
       </c>
       <c r="O9" s="18" t="s"/>
@@ -1676,7 +1676,7 @@
       <c r="L10" s="14" t="s"/>
       <c r="M10" s="14" t="s"/>
       <c r="N10" s="14" t="str">
-        <f>=IF(L10="","",20+L10*5)</f>
+        <f>IF(L10="","",20+L10*5)</f>
         <v/>
       </c>
       <c r="O10" s="18" t="s"/>
@@ -1704,7 +1704,7 @@
       <c r="L11" s="14" t="s"/>
       <c r="M11" s="14" t="s"/>
       <c r="N11" s="14" t="str">
-        <f>=IF(L11="","",20+L11*5)</f>
+        <f>IF(L11="","",20+L11*5)</f>
         <v/>
       </c>
       <c r="O11" s="18" t="s"/>
@@ -1732,7 +1732,7 @@
       <c r="L12" s="14" t="s"/>
       <c r="M12" s="14" t="s"/>
       <c r="N12" s="14" t="str">
-        <f>=IF(L12="","",20+L12*5)</f>
+        <f>IF(L12="","",20+L12*5)</f>
         <v/>
       </c>
       <c r="O12" s="18" t="s"/>
@@ -1760,7 +1760,7 @@
       <c r="L13" s="14" t="s"/>
       <c r="M13" s="14" t="s"/>
       <c r="N13" s="14" t="str">
-        <f>=IF(L13="","",20+L13*5)</f>
+        <f>IF(L13="","",20+L13*5)</f>
         <v/>
       </c>
       <c r="O13" s="18" t="s"/>
@@ -1788,7 +1788,7 @@
       <c r="L14" s="14" t="s"/>
       <c r="M14" s="14" t="s"/>
       <c r="N14" s="14" t="str">
-        <f>=IF(L14="","",20+L14*5)</f>
+        <f>IF(L14="","",20+L14*5)</f>
         <v/>
       </c>
       <c r="O14" s="18" t="s"/>
@@ -1816,7 +1816,7 @@
       <c r="L15" s="14" t="s"/>
       <c r="M15" s="14" t="s"/>
       <c r="N15" s="14" t="str">
-        <f>=IF(L15="","",20+L15*5)</f>
+        <f>IF(L15="","",20+L15*5)</f>
         <v/>
       </c>
       <c r="O15" s="18" t="s"/>
@@ -1844,7 +1844,7 @@
       <c r="L16" s="14" t="s"/>
       <c r="M16" s="14" t="s"/>
       <c r="N16" s="14" t="str">
-        <f>=IF(L16="","",20+L16*5)</f>
+        <f>IF(L16="","",20+L16*5)</f>
         <v/>
       </c>
       <c r="O16" s="18" t="s"/>
@@ -1872,7 +1872,7 @@
       <c r="L17" s="14" t="s"/>
       <c r="M17" s="14" t="s"/>
       <c r="N17" s="14" t="str">
-        <f>=IF(L17="","",20+L17*5)</f>
+        <f>IF(L17="","",20+L17*5)</f>
         <v/>
       </c>
       <c r="O17" s="18" t="s"/>
@@ -1900,7 +1900,7 @@
       <c r="L18" s="14" t="s"/>
       <c r="M18" s="14" t="s"/>
       <c r="N18" s="14" t="str">
-        <f>=IF(L18="","",20+L18*5)</f>
+        <f>IF(L18="","",20+L18*5)</f>
         <v/>
       </c>
       <c r="O18" s="18" t="s"/>
@@ -1928,7 +1928,7 @@
       <c r="L19" s="14" t="s"/>
       <c r="M19" s="14" t="s"/>
       <c r="N19" s="14" t="str">
-        <f>=IF(L19="","",20+L19*5)</f>
+        <f>IF(L19="","",20+L19*5)</f>
         <v/>
       </c>
       <c r="O19" s="18" t="s"/>
@@ -1956,7 +1956,7 @@
       <c r="L20" s="14" t="s"/>
       <c r="M20" s="14" t="s"/>
       <c r="N20" s="14" t="str">
-        <f>=IF(L20="","",20+L20*5)</f>
+        <f>IF(L20="","",20+L20*5)</f>
         <v/>
       </c>
       <c r="O20" s="18" t="s"/>
@@ -1984,7 +1984,7 @@
       <c r="L21" s="14" t="s"/>
       <c r="M21" s="14" t="s"/>
       <c r="N21" s="14" t="str">
-        <f>=IF(L21="","",20+L21*5)</f>
+        <f>IF(L21="","",20+L21*5)</f>
         <v/>
       </c>
       <c r="O21" s="18" t="s"/>
@@ -2012,7 +2012,7 @@
       <c r="L22" s="14" t="s"/>
       <c r="M22" s="14" t="s"/>
       <c r="N22" s="14" t="str">
-        <f>=IF(L22="","",20+L22*5)</f>
+        <f>IF(L22="","",20+L22*5)</f>
         <v/>
       </c>
       <c r="O22" s="18" t="s"/>
@@ -2040,7 +2040,7 @@
       <c r="L23" s="14" t="s"/>
       <c r="M23" s="14" t="s"/>
       <c r="N23" s="14" t="str">
-        <f>=IF(L23="","",20+L23*5)</f>
+        <f>IF(L23="","",20+L23*5)</f>
         <v/>
       </c>
       <c r="O23" s="18" t="s"/>
@@ -2068,7 +2068,7 @@
       <c r="L24" s="14" t="s"/>
       <c r="M24" s="14" t="s"/>
       <c r="N24" s="14" t="str">
-        <f>=IF(L24="","",20+L24*5)</f>
+        <f>IF(L24="","",20+L24*5)</f>
         <v/>
       </c>
       <c r="O24" s="18" t="s"/>
@@ -2096,7 +2096,7 @@
       <c r="L25" s="14" t="s"/>
       <c r="M25" s="14" t="s"/>
       <c r="N25" s="14" t="str">
-        <f>=IF(L25="","",20+L25*5)</f>
+        <f>IF(L25="","",20+L25*5)</f>
         <v/>
       </c>
       <c r="O25" s="18" t="s"/>
@@ -2124,7 +2124,7 @@
       <c r="L26" s="14" t="s"/>
       <c r="M26" s="14" t="s"/>
       <c r="N26" s="14" t="str">
-        <f>=IF(L26="","",20+L26*5)</f>
+        <f>IF(L26="","",20+L26*5)</f>
         <v/>
       </c>
       <c r="O26" s="18" t="s"/>
@@ -2152,7 +2152,7 @@
       <c r="L27" s="14" t="s"/>
       <c r="M27" s="14" t="s"/>
       <c r="N27" s="14" t="str">
-        <f>=IF(L27="","",20+L27*5)</f>
+        <f>IF(L27="","",20+L27*5)</f>
         <v/>
       </c>
       <c r="O27" s="18" t="s"/>
@@ -2180,7 +2180,7 @@
       <c r="L28" s="14" t="s"/>
       <c r="M28" s="14" t="s"/>
       <c r="N28" s="14" t="str">
-        <f>=IF(L28="","",20+L28*5)</f>
+        <f>IF(L28="","",20+L28*5)</f>
         <v/>
       </c>
       <c r="O28" s="18" t="s"/>
@@ -2208,7 +2208,7 @@
       <c r="L29" s="14" t="s"/>
       <c r="M29" s="14" t="s"/>
       <c r="N29" s="14" t="str">
-        <f>=IF(L29="","",20+L29*5)</f>
+        <f>IF(L29="","",20+L29*5)</f>
         <v/>
       </c>
       <c r="O29" s="18" t="s"/>
@@ -2236,7 +2236,7 @@
       <c r="L30" s="14" t="s"/>
       <c r="M30" s="14" t="s"/>
       <c r="N30" s="14" t="str">
-        <f>=IF(L30="","",20+L30*5)</f>
+        <f>IF(L30="","",20+L30*5)</f>
         <v/>
       </c>
       <c r="O30" s="18" t="s"/>
@@ -2264,7 +2264,7 @@
       <c r="L31" s="14" t="s"/>
       <c r="M31" s="14" t="s"/>
       <c r="N31" s="14" t="str">
-        <f>=IF(L31="","",20+L31*5)</f>
+        <f>IF(L31="","",20+L31*5)</f>
         <v/>
       </c>
       <c r="O31" s="18" t="s"/>
@@ -2292,7 +2292,7 @@
       <c r="L32" s="14" t="s"/>
       <c r="M32" s="14" t="s"/>
       <c r="N32" s="14" t="str">
-        <f>=IF(L32="","",20+L32*5)</f>
+        <f>IF(L32="","",20+L32*5)</f>
         <v/>
       </c>
       <c r="O32" s="18" t="s"/>
@@ -2320,7 +2320,7 @@
       <c r="L33" s="14" t="s"/>
       <c r="M33" s="14" t="s"/>
       <c r="N33" s="14" t="str">
-        <f>=IF(L33="","",20+L33*5)</f>
+        <f>IF(L33="","",20+L33*5)</f>
         <v/>
       </c>
       <c r="O33" s="18" t="s"/>
@@ -2348,7 +2348,7 @@
       <c r="L34" s="14" t="s"/>
       <c r="M34" s="14" t="s"/>
       <c r="N34" s="14" t="str">
-        <f>=IF(L34="","",20+L34*5)</f>
+        <f>IF(L34="","",20+L34*5)</f>
         <v/>
       </c>
       <c r="O34" s="18" t="s"/>
@@ -2376,7 +2376,7 @@
       <c r="L35" s="14" t="s"/>
       <c r="M35" s="14" t="s"/>
       <c r="N35" s="14" t="str">
-        <f>=IF(L35="","",20+L35*5)</f>
+        <f>IF(L35="","",20+L35*5)</f>
         <v/>
       </c>
       <c r="O35" s="18" t="s"/>
@@ -2404,7 +2404,7 @@
       <c r="L36" s="14" t="s"/>
       <c r="M36" s="14" t="s"/>
       <c r="N36" s="14" t="str">
-        <f>=IF(L36="","",20+L36*5)</f>
+        <f>IF(L36="","",20+L36*5)</f>
         <v/>
       </c>
       <c r="O36" s="18" t="s"/>
@@ -2432,7 +2432,7 @@
       <c r="L37" s="14" t="s"/>
       <c r="M37" s="14" t="s"/>
       <c r="N37" s="14" t="str">
-        <f>=IF(L37="","",20+L37*5)</f>
+        <f>IF(L37="","",20+L37*5)</f>
         <v/>
       </c>
       <c r="O37" s="18" t="s"/>
@@ -2460,7 +2460,7 @@
       <c r="L38" s="14" t="s"/>
       <c r="M38" s="14" t="s"/>
       <c r="N38" s="14" t="str">
-        <f>=IF(L38="","",20+L38*5)</f>
+        <f>IF(L38="","",20+L38*5)</f>
         <v/>
       </c>
       <c r="O38" s="18" t="s"/>
@@ -2488,7 +2488,7 @@
       <c r="L39" s="14" t="s"/>
       <c r="M39" s="14" t="s"/>
       <c r="N39" s="14" t="str">
-        <f>=IF(L39="","",20+L39*5)</f>
+        <f>IF(L39="","",20+L39*5)</f>
         <v/>
       </c>
       <c r="O39" s="18" t="s"/>
@@ -2516,7 +2516,7 @@
       <c r="L40" s="14" t="s"/>
       <c r="M40" s="14" t="s"/>
       <c r="N40" s="14" t="str">
-        <f>=IF(L40="","",20+L40*5)</f>
+        <f>IF(L40="","",20+L40*5)</f>
         <v/>
       </c>
       <c r="O40" s="18" t="s"/>
@@ -2544,7 +2544,7 @@
       <c r="L41" s="14" t="s"/>
       <c r="M41" s="14" t="s"/>
       <c r="N41" s="14" t="str">
-        <f>=IF(L41="","",20+L41*5)</f>
+        <f>IF(L41="","",20+L41*5)</f>
         <v/>
       </c>
       <c r="O41" s="18" t="s"/>
@@ -2572,7 +2572,7 @@
       <c r="L42" s="14" t="s"/>
       <c r="M42" s="14" t="s"/>
       <c r="N42" s="14" t="str">
-        <f>=IF(L42="","",20+L42*5)</f>
+        <f>IF(L42="","",20+L42*5)</f>
         <v/>
       </c>
       <c r="O42" s="18" t="s"/>
@@ -2600,7 +2600,7 @@
       <c r="L43" s="14" t="s"/>
       <c r="M43" s="14" t="s"/>
       <c r="N43" s="14" t="str">
-        <f>=IF(L43="","",20+L43*5)</f>
+        <f>IF(L43="","",20+L43*5)</f>
         <v/>
       </c>
       <c r="O43" s="18" t="s"/>
@@ -2628,7 +2628,7 @@
       <c r="L44" s="14" t="s"/>
       <c r="M44" s="14" t="s"/>
       <c r="N44" s="14" t="str">
-        <f>=IF(L44="","",20+L44*5)</f>
+        <f>IF(L44="","",20+L44*5)</f>
         <v/>
       </c>
       <c r="O44" s="18" t="s"/>
@@ -2656,7 +2656,7 @@
       <c r="L45" s="14" t="s"/>
       <c r="M45" s="14" t="s"/>
       <c r="N45" s="14" t="str">
-        <f>=IF(L45="","",20+L45*5)</f>
+        <f>IF(L45="","",20+L45*5)</f>
         <v/>
       </c>
       <c r="O45" s="18" t="s"/>
@@ -2684,7 +2684,7 @@
       <c r="L46" s="14" t="s"/>
       <c r="M46" s="14" t="s"/>
       <c r="N46" s="14" t="str">
-        <f>=IF(L46="","",20+L46*5)</f>
+        <f>IF(L46="","",20+L46*5)</f>
         <v/>
       </c>
       <c r="O46" s="18" t="s"/>
@@ -2712,7 +2712,7 @@
       <c r="L47" s="14" t="s"/>
       <c r="M47" s="14" t="s"/>
       <c r="N47" s="14" t="str">
-        <f>=IF(L47="","",20+L47*5)</f>
+        <f>IF(L47="","",20+L47*5)</f>
         <v/>
       </c>
       <c r="O47" s="18" t="s"/>
@@ -2740,7 +2740,7 @@
       <c r="L48" s="14" t="s"/>
       <c r="M48" s="14" t="s"/>
       <c r="N48" s="14" t="str">
-        <f>=IF(L48="","",20+L48*5)</f>
+        <f>IF(L48="","",20+L48*5)</f>
         <v/>
       </c>
       <c r="O48" s="18" t="s"/>
@@ -2768,7 +2768,7 @@
       <c r="L49" s="14" t="s"/>
       <c r="M49" s="14" t="s"/>
       <c r="N49" s="14" t="str">
-        <f>=IF(L49="","",20+L49*5)</f>
+        <f>IF(L49="","",20+L49*5)</f>
         <v/>
       </c>
       <c r="O49" s="18" t="s"/>
@@ -2796,7 +2796,7 @@
       <c r="L50" s="14" t="s"/>
       <c r="M50" s="14" t="s"/>
       <c r="N50" s="14" t="str">
-        <f>=IF(L50="","",20+L50*5)</f>
+        <f>IF(L50="","",20+L50*5)</f>
         <v/>
       </c>
       <c r="O50" s="18" t="s"/>
@@ -2824,7 +2824,7 @@
       <c r="L51" s="14" t="s"/>
       <c r="M51" s="14" t="s"/>
       <c r="N51" s="14" t="str">
-        <f>=IF(L51="","",20+L51*5)</f>
+        <f>IF(L51="","",20+L51*5)</f>
         <v/>
       </c>
       <c r="O51" s="18" t="s"/>
@@ -2852,7 +2852,7 @@
       <c r="L52" s="14" t="s"/>
       <c r="M52" s="14" t="s"/>
       <c r="N52" s="14" t="str">
-        <f>=IF(L52="","",20+L52*5)</f>
+        <f>IF(L52="","",20+L52*5)</f>
         <v/>
       </c>
       <c r="O52" s="18" t="s"/>
@@ -2880,7 +2880,7 @@
       <c r="L53" s="14" t="s"/>
       <c r="M53" s="14" t="s"/>
       <c r="N53" s="14" t="str">
-        <f>=IF(L53="","",20+L53*5)</f>
+        <f>IF(L53="","",20+L53*5)</f>
         <v/>
       </c>
       <c r="O53" s="18" t="s"/>
@@ -2908,7 +2908,7 @@
       <c r="L54" s="14" t="s"/>
       <c r="M54" s="14" t="s"/>
       <c r="N54" s="14" t="str">
-        <f>=IF(L54="","",20+L54*5)</f>
+        <f>IF(L54="","",20+L54*5)</f>
         <v/>
       </c>
       <c r="O54" s="18" t="s"/>
@@ -2936,7 +2936,7 @@
       <c r="L55" s="14" t="s"/>
       <c r="M55" s="14" t="s"/>
       <c r="N55" s="14" t="str">
-        <f>=IF(L55="","",20+L55*5)</f>
+        <f>IF(L55="","",20+L55*5)</f>
         <v/>
       </c>
       <c r="O55" s="18" t="s"/>
@@ -2964,7 +2964,7 @@
       <c r="L56" s="14" t="s"/>
       <c r="M56" s="14" t="s"/>
       <c r="N56" s="14" t="str">
-        <f>=IF(L56="","",20+L56*5)</f>
+        <f>IF(L56="","",20+L56*5)</f>
         <v/>
       </c>
       <c r="O56" s="18" t="s"/>
@@ -2992,7 +2992,7 @@
       <c r="L57" s="14" t="s"/>
       <c r="M57" s="14" t="s"/>
       <c r="N57" s="14" t="str">
-        <f>=IF(L57="","",20+L57*5)</f>
+        <f>IF(L57="","",20+L57*5)</f>
         <v/>
       </c>
       <c r="O57" s="18" t="s"/>
@@ -3020,7 +3020,7 @@
       <c r="L58" s="14" t="s"/>
       <c r="M58" s="14" t="s"/>
       <c r="N58" s="14" t="str">
-        <f>=IF(L58="","",20+L58*5)</f>
+        <f>IF(L58="","",20+L58*5)</f>
         <v/>
       </c>
       <c r="O58" s="18" t="s"/>
@@ -3048,7 +3048,7 @@
       <c r="L59" s="14" t="s"/>
       <c r="M59" s="14" t="s"/>
       <c r="N59" s="14" t="str">
-        <f>=IF(L59="","",20+L59*5)</f>
+        <f>IF(L59="","",20+L59*5)</f>
         <v/>
       </c>
       <c r="O59" s="18" t="s"/>
@@ -3076,7 +3076,7 @@
       <c r="L60" s="14" t="s"/>
       <c r="M60" s="14" t="s"/>
       <c r="N60" s="14" t="str">
-        <f>=IF(L60="","",20+L60*5)</f>
+        <f>IF(L60="","",20+L60*5)</f>
         <v/>
       </c>
       <c r="O60" s="18" t="s"/>
@@ -3104,7 +3104,7 @@
       <c r="L61" s="14" t="s"/>
       <c r="M61" s="14" t="s"/>
       <c r="N61" s="14" t="str">
-        <f>=IF(L61="","",20+L61*5)</f>
+        <f>IF(L61="","",20+L61*5)</f>
         <v/>
       </c>
       <c r="O61" s="18" t="s"/>
@@ -3132,7 +3132,7 @@
       <c r="L62" s="14" t="s"/>
       <c r="M62" s="14" t="s"/>
       <c r="N62" s="14" t="str">
-        <f>=IF(L62="","",20+L62*5)</f>
+        <f>IF(L62="","",20+L62*5)</f>
         <v/>
       </c>
       <c r="O62" s="18" t="s"/>
@@ -3160,7 +3160,7 @@
       <c r="L63" s="14" t="s"/>
       <c r="M63" s="14" t="s"/>
       <c r="N63" s="14" t="str">
-        <f>=IF(L63="","",20+L63*5)</f>
+        <f>IF(L63="","",20+L63*5)</f>
         <v/>
       </c>
       <c r="O63" s="18" t="s"/>
@@ -3188,7 +3188,7 @@
       <c r="L64" s="14" t="s"/>
       <c r="M64" s="14" t="s"/>
       <c r="N64" s="14" t="str">
-        <f>=IF(L64="","",20+L64*5)</f>
+        <f>IF(L64="","",20+L64*5)</f>
         <v/>
       </c>
       <c r="O64" s="18" t="s"/>
@@ -3216,7 +3216,7 @@
       <c r="L65" s="14" t="s"/>
       <c r="M65" s="14" t="s"/>
       <c r="N65" s="14" t="str">
-        <f>=IF(L65="","",20+L65*5)</f>
+        <f>IF(L65="","",20+L65*5)</f>
         <v/>
       </c>
       <c r="O65" s="18" t="s"/>
@@ -3244,7 +3244,7 @@
       <c r="L66" s="14" t="s"/>
       <c r="M66" s="14" t="s"/>
       <c r="N66" s="14" t="str">
-        <f>=IF(L66="","",20+L66*5)</f>
+        <f>IF(L66="","",20+L66*5)</f>
         <v/>
       </c>
       <c r="O66" s="18" t="s"/>
@@ -3272,7 +3272,7 @@
       <c r="L67" s="14" t="s"/>
       <c r="M67" s="14" t="s"/>
       <c r="N67" s="14" t="str">
-        <f>=IF(L67="","",20+L67*5)</f>
+        <f>IF(L67="","",20+L67*5)</f>
         <v/>
       </c>
       <c r="O67" s="18" t="s"/>
@@ -3300,7 +3300,7 @@
       <c r="L68" s="14" t="s"/>
       <c r="M68" s="14" t="s"/>
       <c r="N68" s="14" t="str">
-        <f>=IF(L68="","",20+L68*5)</f>
+        <f>IF(L68="","",20+L68*5)</f>
         <v/>
       </c>
       <c r="O68" s="18" t="s"/>
@@ -3328,7 +3328,7 @@
       <c r="L69" s="14" t="s"/>
       <c r="M69" s="14" t="s"/>
       <c r="N69" s="14" t="str">
-        <f>=IF(L69="","",20+L69*5)</f>
+        <f>IF(L69="","",20+L69*5)</f>
         <v/>
       </c>
       <c r="O69" s="18" t="s"/>
@@ -3356,7 +3356,7 @@
       <c r="L70" s="14" t="s"/>
       <c r="M70" s="14" t="s"/>
       <c r="N70" s="14" t="str">
-        <f>=IF(L70="","",20+L70*5)</f>
+        <f>IF(L70="","",20+L70*5)</f>
         <v/>
       </c>
       <c r="O70" s="18" t="s"/>
@@ -3384,7 +3384,7 @@
       <c r="L71" s="14" t="s"/>
       <c r="M71" s="14" t="s"/>
       <c r="N71" s="14" t="str">
-        <f>=IF(L71="","",20+L71*5)</f>
+        <f>IF(L71="","",20+L71*5)</f>
         <v/>
       </c>
       <c r="O71" s="18" t="s"/>
@@ -3412,7 +3412,7 @@
       <c r="L72" s="14" t="s"/>
       <c r="M72" s="14" t="s"/>
       <c r="N72" s="14" t="str">
-        <f>=IF(L72="","",20+L72*5)</f>
+        <f>IF(L72="","",20+L72*5)</f>
         <v/>
       </c>
       <c r="O72" s="18" t="s"/>
@@ -3440,7 +3440,7 @@
       <c r="L73" s="14" t="s"/>
       <c r="M73" s="14" t="s"/>
       <c r="N73" s="14" t="str">
-        <f>=IF(L73="","",20+L73*5)</f>
+        <f>IF(L73="","",20+L73*5)</f>
         <v/>
       </c>
       <c r="O73" s="18" t="s"/>
@@ -3468,7 +3468,7 @@
       <c r="L74" s="14" t="s"/>
       <c r="M74" s="14" t="s"/>
       <c r="N74" s="14" t="str">
-        <f>=IF(L74="","",20+L74*5)</f>
+        <f>IF(L74="","",20+L74*5)</f>
         <v/>
       </c>
       <c r="O74" s="18" t="s"/>
@@ -3496,7 +3496,7 @@
       <c r="L75" s="14" t="s"/>
       <c r="M75" s="14" t="s"/>
       <c r="N75" s="14" t="str">
-        <f>=IF(L75="","",20+L75*5)</f>
+        <f>IF(L75="","",20+L75*5)</f>
         <v/>
       </c>
       <c r="O75" s="18" t="s"/>
@@ -3524,7 +3524,7 @@
       <c r="L76" s="14" t="s"/>
       <c r="M76" s="14" t="s"/>
       <c r="N76" s="14" t="str">
-        <f>=IF(L76="","",20+L76*5)</f>
+        <f>IF(L76="","",20+L76*5)</f>
         <v/>
       </c>
       <c r="O76" s="18" t="s"/>
@@ -3552,7 +3552,7 @@
       <c r="L77" s="14" t="s"/>
       <c r="M77" s="14" t="s"/>
       <c r="N77" s="14" t="str">
-        <f>=IF(L77="","",20+L77*5)</f>
+        <f>IF(L77="","",20+L77*5)</f>
         <v/>
       </c>
       <c r="O77" s="18" t="s"/>
@@ -3580,7 +3580,7 @@
       <c r="L78" s="14" t="s"/>
       <c r="M78" s="14" t="s"/>
       <c r="N78" s="14" t="str">
-        <f>=IF(L78="","",20+L78*5)</f>
+        <f>IF(L78="","",20+L78*5)</f>
         <v/>
       </c>
       <c r="O78" s="18" t="s"/>
@@ -3608,7 +3608,7 @@
       <c r="L79" s="14" t="s"/>
       <c r="M79" s="14" t="s"/>
       <c r="N79" s="14" t="str">
-        <f>=IF(L79="","",20+L79*5)</f>
+        <f>IF(L79="","",20+L79*5)</f>
         <v/>
       </c>
       <c r="O79" s="18" t="s"/>
@@ -3636,7 +3636,7 @@
       <c r="L80" s="14" t="s"/>
       <c r="M80" s="14" t="s"/>
       <c r="N80" s="14" t="str">
-        <f>=IF(L80="","",20+L80*5)</f>
+        <f>IF(L80="","",20+L80*5)</f>
         <v/>
       </c>
       <c r="O80" s="18" t="s"/>
@@ -3664,7 +3664,7 @@
       <c r="L81" s="14" t="s"/>
       <c r="M81" s="14" t="s"/>
       <c r="N81" s="14" t="str">
-        <f>=IF(L81="","",20+L81*5)</f>
+        <f>IF(L81="","",20+L81*5)</f>
         <v/>
       </c>
       <c r="O81" s="18" t="s"/>
@@ -3692,7 +3692,7 @@
       <c r="L82" s="14" t="s"/>
       <c r="M82" s="14" t="s"/>
       <c r="N82" s="14" t="str">
-        <f>=IF(L82="","",20+L82*5)</f>
+        <f>IF(L82="","",20+L82*5)</f>
         <v/>
       </c>
       <c r="O82" s="18" t="s"/>
@@ -3720,7 +3720,7 @@
       <c r="L83" s="14" t="s"/>
       <c r="M83" s="14" t="s"/>
       <c r="N83" s="14" t="str">
-        <f>=IF(L83="","",20+L83*5)</f>
+        <f>IF(L83="","",20+L83*5)</f>
         <v/>
       </c>
       <c r="O83" s="18" t="s"/>
@@ -3748,7 +3748,7 @@
       <c r="L84" s="14" t="s"/>
       <c r="M84" s="14" t="s"/>
       <c r="N84" s="14" t="str">
-        <f>=IF(L84="","",20+L84*5)</f>
+        <f>IF(L84="","",20+L84*5)</f>
         <v/>
       </c>
       <c r="O84" s="18" t="s"/>
@@ -3776,7 +3776,7 @@
       <c r="L85" s="14" t="s"/>
       <c r="M85" s="14" t="s"/>
       <c r="N85" s="14" t="str">
-        <f>=IF(L85="","",20+L85*5)</f>
+        <f>IF(L85="","",20+L85*5)</f>
         <v/>
       </c>
       <c r="O85" s="18" t="s"/>
@@ -3804,7 +3804,7 @@
       <c r="L86" s="14" t="s"/>
       <c r="M86" s="14" t="s"/>
       <c r="N86" s="14" t="str">
-        <f>=IF(L86="","",20+L86*5)</f>
+        <f>IF(L86="","",20+L86*5)</f>
         <v/>
       </c>
       <c r="O86" s="18" t="s"/>
@@ -3832,7 +3832,7 @@
       <c r="L87" s="14" t="s"/>
       <c r="M87" s="14" t="s"/>
       <c r="N87" s="14" t="str">
-        <f>=IF(L87="","",20+L87*5)</f>
+        <f>IF(L87="","",20+L87*5)</f>
         <v/>
       </c>
       <c r="O87" s="18" t="s"/>
@@ -3860,7 +3860,7 @@
       <c r="L88" s="14" t="s"/>
       <c r="M88" s="14" t="s"/>
       <c r="N88" s="14" t="str">
-        <f>=IF(L88="","",20+L88*5)</f>
+        <f>IF(L88="","",20+L88*5)</f>
         <v/>
       </c>
       <c r="O88" s="18" t="s"/>
@@ -3888,7 +3888,7 @@
       <c r="L89" s="14" t="s"/>
       <c r="M89" s="14" t="s"/>
       <c r="N89" s="14" t="str">
-        <f>=IF(L89="","",20+L89*5)</f>
+        <f>IF(L89="","",20+L89*5)</f>
         <v/>
       </c>
       <c r="O89" s="18" t="s"/>
@@ -3916,7 +3916,7 @@
       <c r="L90" s="14" t="s"/>
       <c r="M90" s="14" t="s"/>
       <c r="N90" s="14" t="str">
-        <f>=IF(L90="","",20+L90*5)</f>
+        <f>IF(L90="","",20+L90*5)</f>
         <v/>
       </c>
       <c r="O90" s="18" t="s"/>
@@ -3944,7 +3944,7 @@
       <c r="L91" s="14" t="s"/>
       <c r="M91" s="14" t="s"/>
       <c r="N91" s="14" t="str">
-        <f>=IF(L91="","",20+L91*5)</f>
+        <f>IF(L91="","",20+L91*5)</f>
         <v/>
       </c>
       <c r="O91" s="18" t="s"/>
@@ -3972,7 +3972,7 @@
       <c r="L92" s="14" t="s"/>
       <c r="M92" s="14" t="s"/>
       <c r="N92" s="14" t="str">
-        <f>=IF(L92="","",20+L92*5)</f>
+        <f>IF(L92="","",20+L92*5)</f>
         <v/>
       </c>
       <c r="O92" s="18" t="s"/>
@@ -4000,7 +4000,7 @@
       <c r="L93" s="14" t="s"/>
       <c r="M93" s="14" t="s"/>
       <c r="N93" s="14" t="str">
-        <f>=IF(L93="","",20+L93*5)</f>
+        <f>IF(L93="","",20+L93*5)</f>
         <v/>
       </c>
       <c r="O93" s="18" t="s"/>
@@ -4028,7 +4028,7 @@
       <c r="L94" s="14" t="s"/>
       <c r="M94" s="14" t="s"/>
       <c r="N94" s="14" t="str">
-        <f>=IF(L94="","",20+L94*5)</f>
+        <f>IF(L94="","",20+L94*5)</f>
         <v/>
       </c>
       <c r="O94" s="18" t="s"/>
@@ -4056,7 +4056,7 @@
       <c r="L95" s="14" t="s"/>
       <c r="M95" s="14" t="s"/>
       <c r="N95" s="14" t="str">
-        <f>=IF(L95="","",20+L95*5)</f>
+        <f>IF(L95="","",20+L95*5)</f>
         <v/>
       </c>
       <c r="O95" s="18" t="s"/>
@@ -4084,7 +4084,7 @@
       <c r="L96" s="14" t="s"/>
       <c r="M96" s="14" t="s"/>
       <c r="N96" s="14" t="str">
-        <f>=IF(L96="","",20+L96*5)</f>
+        <f>IF(L96="","",20+L96*5)</f>
         <v/>
       </c>
       <c r="O96" s="18" t="s"/>
@@ -4112,7 +4112,7 @@
       <c r="L97" s="14" t="s"/>
       <c r="M97" s="14" t="s"/>
       <c r="N97" s="14" t="str">
-        <f>=IF(L97="","",20+L97*5)</f>
+        <f>IF(L97="","",20+L97*5)</f>
         <v/>
       </c>
       <c r="O97" s="18" t="s"/>
@@ -4140,7 +4140,7 @@
       <c r="L98" s="14" t="s"/>
       <c r="M98" s="14" t="s"/>
       <c r="N98" s="14" t="str">
-        <f>=IF(L98="","",20+L98*5)</f>
+        <f>IF(L98="","",20+L98*5)</f>
         <v/>
       </c>
       <c r="O98" s="18" t="s"/>
@@ -4168,7 +4168,7 @@
       <c r="L99" s="14" t="s"/>
       <c r="M99" s="14" t="s"/>
       <c r="N99" s="14" t="str">
-        <f>=IF(L99="","",20+L99*5)</f>
+        <f>IF(L99="","",20+L99*5)</f>
         <v/>
       </c>
       <c r="O99" s="18" t="s"/>
@@ -4196,7 +4196,7 @@
       <c r="L100" s="14" t="s"/>
       <c r="M100" s="14" t="s"/>
       <c r="N100" s="14" t="str">
-        <f>=IF(L100="","",20+L100*5)</f>
+        <f>IF(L100="","",20+L100*5)</f>
         <v/>
       </c>
       <c r="O100" s="18" t="s"/>
@@ -4224,7 +4224,7 @@
       <c r="L101" s="14" t="s"/>
       <c r="M101" s="14" t="s"/>
       <c r="N101" s="14" t="str">
-        <f>=IF(L101="","",20+L101*5)</f>
+        <f>IF(L101="","",20+L101*5)</f>
         <v/>
       </c>
       <c r="O101" s="18" t="s"/>
@@ -4252,7 +4252,7 @@
       <c r="L102" s="14" t="s"/>
       <c r="M102" s="14" t="s"/>
       <c r="N102" s="14" t="str">
-        <f>=IF(L102="","",20+L102*5)</f>
+        <f>IF(L102="","",20+L102*5)</f>
         <v/>
       </c>
       <c r="O102" s="18" t="s"/>
@@ -4280,7 +4280,7 @@
       <c r="L103" s="14" t="s"/>
       <c r="M103" s="14" t="s"/>
       <c r="N103" s="14" t="str">
-        <f>=IF(L103="","",20+L103*5)</f>
+        <f>IF(L103="","",20+L103*5)</f>
         <v/>
       </c>
       <c r="O103" s="18" t="s"/>
@@ -4308,7 +4308,7 @@
       <c r="L104" s="14" t="s"/>
       <c r="M104" s="14" t="s"/>
       <c r="N104" s="14" t="str">
-        <f>=IF(L104="","",20+L104*5)</f>
+        <f>IF(L104="","",20+L104*5)</f>
         <v/>
       </c>
       <c r="O104" s="18" t="s"/>
@@ -4336,7 +4336,7 @@
       <c r="L105" s="14" t="s"/>
       <c r="M105" s="14" t="s"/>
       <c r="N105" s="14" t="str">
-        <f>=IF(L105="","",20+L105*5)</f>
+        <f>IF(L105="","",20+L105*5)</f>
         <v/>
       </c>
       <c r="O105" s="18" t="s"/>
@@ -4364,7 +4364,7 @@
       <c r="L106" s="14" t="s"/>
       <c r="M106" s="14" t="s"/>
       <c r="N106" s="14" t="str">
-        <f>=IF(L106="","",20+L106*5)</f>
+        <f>IF(L106="","",20+L106*5)</f>
         <v/>
       </c>
       <c r="O106" s="18" t="s"/>
@@ -4392,7 +4392,7 @@
       <c r="L107" s="14" t="s"/>
       <c r="M107" s="14" t="s"/>
       <c r="N107" s="14" t="str">
-        <f>=IF(L107="","",20+L107*5)</f>
+        <f>IF(L107="","",20+L107*5)</f>
         <v/>
       </c>
       <c r="O107" s="18" t="s"/>
@@ -4420,7 +4420,7 @@
       <c r="L108" s="14" t="s"/>
       <c r="M108" s="14" t="s"/>
       <c r="N108" s="14" t="str">
-        <f>=IF(L108="","",20+L108*5)</f>
+        <f>IF(L108="","",20+L108*5)</f>
         <v/>
       </c>
       <c r="O108" s="18" t="s"/>
@@ -4448,7 +4448,7 @@
       <c r="L109" s="14" t="s"/>
       <c r="M109" s="14" t="s"/>
       <c r="N109" s="14" t="str">
-        <f>=IF(L109="","",20+L109*5)</f>
+        <f>IF(L109="","",20+L109*5)</f>
         <v/>
       </c>
       <c r="O109" s="18" t="s"/>
@@ -4476,7 +4476,7 @@
       <c r="L110" s="14" t="s"/>
       <c r="M110" s="14" t="s"/>
       <c r="N110" s="14" t="str">
-        <f>=IF(L110="","",20+L110*5)</f>
+        <f>IF(L110="","",20+L110*5)</f>
         <v/>
       </c>
       <c r="O110" s="18" t="s"/>
@@ -4504,7 +4504,7 @@
       <c r="L111" s="14" t="s"/>
       <c r="M111" s="14" t="s"/>
       <c r="N111" s="14" t="str">
-        <f>=IF(L111="","",20+L111*5)</f>
+        <f>IF(L111="","",20+L111*5)</f>
         <v/>
       </c>
       <c r="O111" s="18" t="s"/>
@@ -4532,7 +4532,7 @@
       <c r="L112" s="14" t="s"/>
       <c r="M112" s="14" t="s"/>
       <c r="N112" s="14" t="str">
-        <f>=IF(L112="","",20+L112*5)</f>
+        <f>IF(L112="","",20+L112*5)</f>
         <v/>
       </c>
       <c r="O112" s="18" t="s"/>
@@ -4560,7 +4560,7 @@
       <c r="L113" s="14" t="s"/>
       <c r="M113" s="14" t="s"/>
       <c r="N113" s="14" t="str">
-        <f>=IF(L113="","",20+L113*5)</f>
+        <f>IF(L113="","",20+L113*5)</f>
         <v/>
       </c>
       <c r="O113" s="18" t="s"/>
@@ -4588,7 +4588,7 @@
       <c r="L114" s="14" t="s"/>
       <c r="M114" s="14" t="s"/>
       <c r="N114" s="14" t="str">
-        <f>=IF(L114="","",20+L114*5)</f>
+        <f>IF(L114="","",20+L114*5)</f>
         <v/>
       </c>
       <c r="O114" s="18" t="s"/>
@@ -4616,7 +4616,7 @@
       <c r="L115" s="14" t="s"/>
       <c r="M115" s="14" t="s"/>
       <c r="N115" s="14" t="str">
-        <f>=IF(L115="","",20+L115*5)</f>
+        <f>IF(L115="","",20+L115*5)</f>
         <v/>
       </c>
       <c r="O115" s="18" t="s"/>
@@ -4644,7 +4644,7 @@
       <c r="L116" s="14" t="s"/>
       <c r="M116" s="14" t="s"/>
       <c r="N116" s="14" t="str">
-        <f>=IF(L116="","",20+L116*5)</f>
+        <f>IF(L116="","",20+L116*5)</f>
         <v/>
       </c>
       <c r="O116" s="18" t="s"/>
@@ -4672,7 +4672,7 @@
       <c r="L117" s="14" t="s"/>
       <c r="M117" s="14" t="s"/>
       <c r="N117" s="14" t="str">
-        <f>=IF(L117="","",20+L117*5)</f>
+        <f>IF(L117="","",20+L117*5)</f>
         <v/>
       </c>
       <c r="O117" s="18" t="s"/>
@@ -4700,7 +4700,7 @@
       <c r="L118" s="14" t="s"/>
       <c r="M118" s="14" t="s"/>
       <c r="N118" s="14" t="str">
-        <f>=IF(L118="","",20+L118*5)</f>
+        <f>IF(L118="","",20+L118*5)</f>
         <v/>
       </c>
       <c r="O118" s="18" t="s"/>
@@ -4728,7 +4728,7 @@
       <c r="L119" s="14" t="s"/>
       <c r="M119" s="14" t="s"/>
       <c r="N119" s="14" t="str">
-        <f>=IF(L119="","",20+L119*5)</f>
+        <f>IF(L119="","",20+L119*5)</f>
         <v/>
       </c>
       <c r="O119" s="18" t="s"/>
@@ -4756,7 +4756,7 @@
       <c r="L120" s="14" t="s"/>
       <c r="M120" s="14" t="s"/>
       <c r="N120" s="14" t="str">
-        <f>=IF(L120="","",20+L120*5)</f>
+        <f>IF(L120="","",20+L120*5)</f>
         <v/>
       </c>
       <c r="O120" s="18" t="s"/>
@@ -4784,7 +4784,7 @@
       <c r="L121" s="14" t="s"/>
       <c r="M121" s="14" t="s"/>
       <c r="N121" s="14" t="str">
-        <f>=IF(L121="","",20+L121*5)</f>
+        <f>IF(L121="","",20+L121*5)</f>
         <v/>
       </c>
       <c r="O121" s="18" t="s"/>
@@ -4812,7 +4812,7 @@
       <c r="L122" s="14" t="s"/>
       <c r="M122" s="14" t="s"/>
       <c r="N122" s="14" t="str">
-        <f>=IF(L122="","",20+L122*5)</f>
+        <f>IF(L122="","",20+L122*5)</f>
         <v/>
       </c>
       <c r="O122" s="18" t="s"/>
@@ -4840,7 +4840,7 @@
       <c r="L123" s="14" t="s"/>
       <c r="M123" s="14" t="s"/>
       <c r="N123" s="14" t="str">
-        <f>=IF(L123="","",20+L123*5)</f>
+        <f>IF(L123="","",20+L123*5)</f>
         <v/>
       </c>
       <c r="O123" s="18" t="s"/>
@@ -4868,7 +4868,7 @@
       <c r="L124" s="14" t="s"/>
       <c r="M124" s="14" t="s"/>
       <c r="N124" s="14" t="str">
-        <f>=IF(L124="","",20+L124*5)</f>
+        <f>IF(L124="","",20+L124*5)</f>
         <v/>
       </c>
       <c r="O124" s="18" t="s"/>
@@ -4896,7 +4896,7 @@
       <c r="L125" s="14" t="s"/>
       <c r="M125" s="14" t="s"/>
       <c r="N125" s="14" t="str">
-        <f>=IF(L125="","",20+L125*5)</f>
+        <f>IF(L125="","",20+L125*5)</f>
         <v/>
       </c>
       <c r="O125" s="18" t="s"/>
@@ -4924,7 +4924,7 @@
       <c r="L126" s="14" t="s"/>
       <c r="M126" s="14" t="s"/>
       <c r="N126" s="14" t="str">
-        <f>=IF(L126="","",20+L126*5)</f>
+        <f>IF(L126="","",20+L126*5)</f>
         <v/>
       </c>
       <c r="O126" s="18" t="s"/>
@@ -4952,7 +4952,7 @@
       <c r="L127" s="14" t="s"/>
       <c r="M127" s="14" t="s"/>
       <c r="N127" s="14" t="str">
-        <f>=IF(L127="","",20+L127*5)</f>
+        <f>IF(L127="","",20+L127*5)</f>
         <v/>
       </c>
       <c r="O127" s="18" t="s"/>
@@ -4980,7 +4980,7 @@
       <c r="L128" s="14" t="s"/>
       <c r="M128" s="14" t="s"/>
       <c r="N128" s="14" t="str">
-        <f>=IF(L128="","",20+L128*5)</f>
+        <f>IF(L128="","",20+L128*5)</f>
         <v/>
       </c>
       <c r="O128" s="18" t="s"/>
@@ -5008,7 +5008,7 @@
       <c r="L129" s="14" t="s"/>
       <c r="M129" s="14" t="s"/>
       <c r="N129" s="14" t="str">
-        <f>=IF(L129="","",20+L129*5)</f>
+        <f>IF(L129="","",20+L129*5)</f>
         <v/>
       </c>
       <c r="O129" s="18" t="s"/>
@@ -5036,7 +5036,7 @@
       <c r="L130" s="14" t="s"/>
       <c r="M130" s="14" t="s"/>
       <c r="N130" s="14" t="str">
-        <f>=IF(L130="","",20+L130*5)</f>
+        <f>IF(L130="","",20+L130*5)</f>
         <v/>
       </c>
       <c r="O130" s="18" t="s"/>
@@ -5064,7 +5064,7 @@
       <c r="L131" s="14" t="s"/>
       <c r="M131" s="14" t="s"/>
       <c r="N131" s="14" t="str">
-        <f>=IF(L131="","",20+L131*5)</f>
+        <f>IF(L131="","",20+L131*5)</f>
         <v/>
       </c>
       <c r="O131" s="18" t="s"/>
@@ -5092,7 +5092,7 @@
       <c r="L132" s="14" t="s"/>
       <c r="M132" s="14" t="s"/>
       <c r="N132" s="14" t="str">
-        <f>=IF(L132="","",20+L132*5)</f>
+        <f>IF(L132="","",20+L132*5)</f>
         <v/>
       </c>
       <c r="O132" s="18" t="s"/>
@@ -5120,7 +5120,7 @@
       <c r="L133" s="14" t="s"/>
       <c r="M133" s="14" t="s"/>
       <c r="N133" s="14" t="str">
-        <f>=IF(L133="","",20+L133*5)</f>
+        <f>IF(L133="","",20+L133*5)</f>
         <v/>
       </c>
       <c r="O133" s="18" t="s"/>
@@ -5148,7 +5148,7 @@
       <c r="L134" s="14" t="s"/>
       <c r="M134" s="14" t="s"/>
       <c r="N134" s="14" t="str">
-        <f>=IF(L134="","",20+L134*5)</f>
+        <f>IF(L134="","",20+L134*5)</f>
         <v/>
       </c>
       <c r="O134" s="18" t="s"/>
@@ -5176,7 +5176,7 @@
       <c r="L135" s="14" t="s"/>
       <c r="M135" s="14" t="s"/>
       <c r="N135" s="14" t="str">
-        <f>=IF(L135="","",20+L135*5)</f>
+        <f>IF(L135="","",20+L135*5)</f>
         <v/>
       </c>
       <c r="O135" s="18" t="s"/>
@@ -5204,7 +5204,7 @@
       <c r="L136" s="14" t="s"/>
       <c r="M136" s="14" t="s"/>
       <c r="N136" s="14" t="str">
-        <f>=IF(L136="","",20+L136*5)</f>
+        <f>IF(L136="","",20+L136*5)</f>
         <v/>
       </c>
       <c r="O136" s="18" t="s"/>
@@ -5232,7 +5232,7 @@
       <c r="L137" s="14" t="s"/>
       <c r="M137" s="14" t="s"/>
       <c r="N137" s="14" t="str">
-        <f>=IF(L137="","",20+L137*5)</f>
+        <f>IF(L137="","",20+L137*5)</f>
         <v/>
       </c>
       <c r="O137" s="18" t="s"/>
@@ -5260,7 +5260,7 @@
       <c r="L138" s="14" t="s"/>
       <c r="M138" s="14" t="s"/>
       <c r="N138" s="14" t="str">
-        <f>=IF(L138="","",20+L138*5)</f>
+        <f>IF(L138="","",20+L138*5)</f>
         <v/>
       </c>
       <c r="O138" s="18" t="s"/>
@@ -5288,7 +5288,7 @@
       <c r="L139" s="14" t="s"/>
       <c r="M139" s="14" t="s"/>
       <c r="N139" s="14" t="str">
-        <f>=IF(L139="","",20+L139*5)</f>
+        <f>IF(L139="","",20+L139*5)</f>
         <v/>
       </c>
       <c r="O139" s="18" t="s"/>
@@ -5316,7 +5316,7 @@
       <c r="L140" s="14" t="s"/>
       <c r="M140" s="14" t="s"/>
       <c r="N140" s="14" t="str">
-        <f>=IF(L140="","",20+L140*5)</f>
+        <f>IF(L140="","",20+L140*5)</f>
         <v/>
       </c>
       <c r="O140" s="18" t="s"/>
@@ -5344,7 +5344,7 @@
       <c r="L141" s="14" t="s"/>
       <c r="M141" s="14" t="s"/>
       <c r="N141" s="14" t="str">
-        <f>=IF(L141="","",20+L141*5)</f>
+        <f>IF(L141="","",20+L141*5)</f>
         <v/>
       </c>
       <c r="O141" s="18" t="s"/>
@@ -5372,7 +5372,7 @@
       <c r="L142" s="14" t="s"/>
       <c r="M142" s="14" t="s"/>
       <c r="N142" s="14" t="str">
-        <f>=IF(L142="","",20+L142*5)</f>
+        <f>IF(L142="","",20+L142*5)</f>
         <v/>
       </c>
       <c r="O142" s="18" t="s"/>
@@ -5400,7 +5400,7 @@
       <c r="L143" s="14" t="s"/>
       <c r="M143" s="14" t="s"/>
       <c r="N143" s="14" t="str">
-        <f>=IF(L143="","",20+L143*5)</f>
+        <f>IF(L143="","",20+L143*5)</f>
         <v/>
       </c>
       <c r="O143" s="18" t="s"/>
@@ -5428,7 +5428,7 @@
       <c r="L144" s="14" t="s"/>
       <c r="M144" s="14" t="s"/>
       <c r="N144" s="14" t="str">
-        <f>=IF(L144="","",20+L144*5)</f>
+        <f>IF(L144="","",20+L144*5)</f>
         <v/>
       </c>
       <c r="O144" s="18" t="s"/>
@@ -5456,7 +5456,7 @@
       <c r="L145" s="14" t="s"/>
       <c r="M145" s="14" t="s"/>
       <c r="N145" s="14" t="str">
-        <f>=IF(L145="","",20+L145*5)</f>
+        <f>IF(L145="","",20+L145*5)</f>
         <v/>
       </c>
       <c r="O145" s="18" t="s"/>
@@ -5484,7 +5484,7 @@
       <c r="L146" s="14" t="s"/>
       <c r="M146" s="14" t="s"/>
       <c r="N146" s="14" t="str">
-        <f>=IF(L146="","",20+L146*5)</f>
+        <f>IF(L146="","",20+L146*5)</f>
         <v/>
       </c>
       <c r="O146" s="18" t="s"/>
@@ -5512,7 +5512,7 @@
       <c r="L147" s="14" t="s"/>
       <c r="M147" s="14" t="s"/>
       <c r="N147" s="14" t="str">
-        <f>=IF(L147="","",20+L147*5)</f>
+        <f>IF(L147="","",20+L147*5)</f>
         <v/>
       </c>
       <c r="O147" s="18" t="s"/>
@@ -5540,7 +5540,7 @@
       <c r="L148" s="14" t="s"/>
       <c r="M148" s="14" t="s"/>
       <c r="N148" s="14" t="str">
-        <f>=IF(L148="","",20+L148*5)</f>
+        <f>IF(L148="","",20+L148*5)</f>
         <v/>
       </c>
       <c r="O148" s="18" t="s"/>
@@ -5568,7 +5568,7 @@
       <c r="L149" s="14" t="s"/>
       <c r="M149" s="14" t="s"/>
       <c r="N149" s="14" t="str">
-        <f>=IF(L149="","",20+L149*5)</f>
+        <f>IF(L149="","",20+L149*5)</f>
         <v/>
       </c>
       <c r="O149" s="18" t="s"/>
@@ -5596,7 +5596,7 @@
       <c r="L150" s="14" t="s"/>
       <c r="M150" s="14" t="s"/>
       <c r="N150" s="14" t="str">
-        <f>=IF(L150="","",20+L150*5)</f>
+        <f>IF(L150="","",20+L150*5)</f>
         <v/>
       </c>
       <c r="O150" s="18" t="s"/>
@@ -5624,7 +5624,7 @@
       <c r="L151" s="14" t="s"/>
       <c r="M151" s="14" t="s"/>
       <c r="N151" s="14" t="str">
-        <f>=IF(L151="","",20+L151*5)</f>
+        <f>IF(L151="","",20+L151*5)</f>
         <v/>
       </c>
       <c r="O151" s="18" t="s"/>
@@ -5652,7 +5652,7 @@
       <c r="L152" s="14" t="s"/>
       <c r="M152" s="14" t="s"/>
       <c r="N152" s="14" t="str">
-        <f>=IF(L152="","",20+L152*5)</f>
+        <f>IF(L152="","",20+L152*5)</f>
         <v/>
       </c>
       <c r="O152" s="18" t="s"/>
@@ -5680,7 +5680,7 @@
       <c r="L153" s="14" t="s"/>
       <c r="M153" s="14" t="s"/>
       <c r="N153" s="14" t="str">
-        <f>=IF(L153="","",20+L153*5)</f>
+        <f>IF(L153="","",20+L153*5)</f>
         <v/>
       </c>
       <c r="O153" s="18" t="s"/>
@@ -5708,7 +5708,7 @@
       <c r="L154" s="14" t="s"/>
       <c r="M154" s="14" t="s"/>
       <c r="N154" s="14" t="str">
-        <f>=IF(L154="","",20+L154*5)</f>
+        <f>IF(L154="","",20+L154*5)</f>
         <v/>
       </c>
       <c r="O154" s="18" t="s"/>
@@ -5736,7 +5736,7 @@
       <c r="L155" s="14" t="s"/>
       <c r="M155" s="14" t="s"/>
       <c r="N155" s="14" t="str">
-        <f>=IF(L155="","",20+L155*5)</f>
+        <f>IF(L155="","",20+L155*5)</f>
         <v/>
       </c>
       <c r="O155" s="18" t="s"/>
@@ -5764,7 +5764,7 @@
       <c r="L156" s="14" t="s"/>
       <c r="M156" s="14" t="s"/>
       <c r="N156" s="14" t="str">
-        <f>=IF(L156="","",20+L156*5)</f>
+        <f>IF(L156="","",20+L156*5)</f>
         <v/>
       </c>
       <c r="O156" s="18" t="s"/>
@@ -5792,7 +5792,7 @@
       <c r="L157" s="14" t="s"/>
       <c r="M157" s="14" t="s"/>
       <c r="N157" s="14" t="str">
-        <f>=IF(L157="","",20+L157*5)</f>
+        <f>IF(L157="","",20+L157*5)</f>
         <v/>
       </c>
       <c r="O157" s="18" t="s"/>
@@ -5820,7 +5820,7 @@
       <c r="L158" s="14" t="s"/>
       <c r="M158" s="14" t="s"/>
       <c r="N158" s="14" t="str">
-        <f>=IF(L158="","",20+L158*5)</f>
+        <f>IF(L158="","",20+L158*5)</f>
         <v/>
       </c>
       <c r="O158" s="18" t="s"/>
@@ -5848,7 +5848,7 @@
       <c r="L159" s="14" t="s"/>
       <c r="M159" s="14" t="s"/>
       <c r="N159" s="14" t="str">
-        <f>=IF(L159="","",20+L159*5)</f>
+        <f>IF(L159="","",20+L159*5)</f>
         <v/>
       </c>
       <c r="O159" s="18" t="s"/>
@@ -5876,7 +5876,7 @@
       <c r="L160" s="14" t="s"/>
       <c r="M160" s="14" t="s"/>
       <c r="N160" s="14" t="str">
-        <f>=IF(L160="","",20+L160*5)</f>
+        <f>IF(L160="","",20+L160*5)</f>
         <v/>
       </c>
       <c r="O160" s="18" t="s"/>
@@ -5904,7 +5904,7 @@
       <c r="L161" s="14" t="s"/>
       <c r="M161" s="14" t="s"/>
       <c r="N161" s="14" t="str">
-        <f>=IF(L161="","",20+L161*5)</f>
+        <f>IF(L161="","",20+L161*5)</f>
         <v/>
       </c>
       <c r="O161" s="18" t="s"/>
@@ -5932,7 +5932,7 @@
       <c r="L162" s="14" t="s"/>
       <c r="M162" s="14" t="s"/>
       <c r="N162" s="14" t="str">
-        <f>=IF(L162="","",20+L162*5)</f>
+        <f>IF(L162="","",20+L162*5)</f>
         <v/>
       </c>
       <c r="O162" s="18" t="s"/>
@@ -5960,7 +5960,7 @@
       <c r="L163" s="14" t="s"/>
       <c r="M163" s="14" t="s"/>
       <c r="N163" s="14" t="str">
-        <f>=IF(L163="","",20+L163*5)</f>
+        <f>IF(L163="","",20+L163*5)</f>
         <v/>
       </c>
       <c r="O163" s="18" t="s"/>
@@ -5988,7 +5988,7 @@
       <c r="L164" s="14" t="s"/>
       <c r="M164" s="14" t="s"/>
       <c r="N164" s="14" t="str">
-        <f>=IF(L164="","",20+L164*5)</f>
+        <f>IF(L164="","",20+L164*5)</f>
         <v/>
       </c>
       <c r="O164" s="18" t="s"/>
@@ -6016,7 +6016,7 @@
       <c r="L165" s="14" t="s"/>
       <c r="M165" s="14" t="s"/>
       <c r="N165" s="14" t="str">
-        <f>=IF(L165="","",20+L165*5)</f>
+        <f>IF(L165="","",20+L165*5)</f>
         <v/>
       </c>
       <c r="O165" s="18" t="s"/>
@@ -6044,7 +6044,7 @@
       <c r="L166" s="14" t="s"/>
       <c r="M166" s="14" t="s"/>
       <c r="N166" s="14" t="str">
-        <f>=IF(L166="","",20+L166*5)</f>
+        <f>IF(L166="","",20+L166*5)</f>
         <v/>
       </c>
       <c r="O166" s="18" t="s"/>
@@ -6072,7 +6072,7 @@
       <c r="L167" s="14" t="s"/>
       <c r="M167" s="14" t="s"/>
       <c r="N167" s="14" t="str">
-        <f>=IF(L167="","",20+L167*5)</f>
+        <f>IF(L167="","",20+L167*5)</f>
         <v/>
       </c>
       <c r="O167" s="18" t="s"/>
@@ -6100,7 +6100,7 @@
       <c r="L168" s="14" t="s"/>
       <c r="M168" s="14" t="s"/>
       <c r="N168" s="14" t="str">
-        <f>=IF(L168="","",20+L168*5)</f>
+        <f>IF(L168="","",20+L168*5)</f>
         <v/>
       </c>
       <c r="O168" s="18" t="s"/>
@@ -6128,7 +6128,7 @@
       <c r="L169" s="14" t="s"/>
       <c r="M169" s="14" t="s"/>
       <c r="N169" s="14" t="str">
-        <f>=IF(L169="","",20+L169*5)</f>
+        <f>IF(L169="","",20+L169*5)</f>
         <v/>
       </c>
       <c r="O169" s="18" t="s"/>
@@ -6156,7 +6156,7 @@
       <c r="L170" s="14" t="s"/>
       <c r="M170" s="14" t="s"/>
       <c r="N170" s="14" t="str">
-        <f>=IF(L170="","",20+L170*5)</f>
+        <f>IF(L170="","",20+L170*5)</f>
         <v/>
       </c>
       <c r="O170" s="18" t="s"/>
@@ -6184,7 +6184,7 @@
       <c r="L171" s="14" t="s"/>
       <c r="M171" s="14" t="s"/>
       <c r="N171" s="14" t="str">
-        <f>=IF(L171="","",20+L171*5)</f>
+        <f>IF(L171="","",20+L171*5)</f>
         <v/>
       </c>
       <c r="O171" s="18" t="s"/>
@@ -6212,7 +6212,7 @@
       <c r="L172" s="14" t="s"/>
       <c r="M172" s="14" t="s"/>
       <c r="N172" s="14" t="str">
-        <f>=IF(L172="","",20+L172*5)</f>
+        <f>IF(L172="","",20+L172*5)</f>
         <v/>
       </c>
       <c r="O172" s="18" t="s"/>
@@ -6240,7 +6240,7 @@
       <c r="L173" s="14" t="s"/>
       <c r="M173" s="14" t="s"/>
       <c r="N173" s="14" t="str">
-        <f>=IF(L173="","",20+L173*5)</f>
+        <f>IF(L173="","",20+L173*5)</f>
         <v/>
       </c>
       <c r="O173" s="18" t="s"/>
@@ -6268,7 +6268,7 @@
       <c r="L174" s="14" t="s"/>
       <c r="M174" s="14" t="s"/>
       <c r="N174" s="14" t="str">
-        <f>=IF(L174="","",20+L174*5)</f>
+        <f>IF(L174="","",20+L174*5)</f>
         <v/>
       </c>
       <c r="O174" s="18" t="s"/>
@@ -6296,7 +6296,7 @@
       <c r="L175" s="14" t="s"/>
       <c r="M175" s="14" t="s"/>
       <c r="N175" s="14" t="str">
-        <f>=IF(L175="","",20+L175*5)</f>
+        <f>IF(L175="","",20+L175*5)</f>
         <v/>
       </c>
       <c r="O175" s="18" t="s"/>
@@ -6324,7 +6324,7 @@
       <c r="L176" s="14" t="s"/>
       <c r="M176" s="14" t="s"/>
       <c r="N176" s="14" t="str">
-        <f>=IF(L176="","",20+L176*5)</f>
+        <f>IF(L176="","",20+L176*5)</f>
         <v/>
       </c>
       <c r="O176" s="18" t="s"/>
@@ -6352,7 +6352,7 @@
       <c r="L177" s="14" t="s"/>
       <c r="M177" s="14" t="s"/>
       <c r="N177" s="14" t="str">
-        <f>=IF(L177="","",20+L177*5)</f>
+        <f>IF(L177="","",20+L177*5)</f>
         <v/>
       </c>
       <c r="O177" s="18" t="s"/>
@@ -6380,7 +6380,7 @@
       <c r="L178" s="14" t="s"/>
       <c r="M178" s="14" t="s"/>
       <c r="N178" s="14" t="str">
-        <f>=IF(L178="","",20+L178*5)</f>
+        <f>IF(L178="","",20+L178*5)</f>
         <v/>
       </c>
       <c r="O178" s="18" t="s"/>
@@ -6408,7 +6408,7 @@
       <c r="L179" s="14" t="s"/>
       <c r="M179" s="14" t="s"/>
       <c r="N179" s="14" t="str">
-        <f>=IF(L179="","",20+L179*5)</f>
+        <f>IF(L179="","",20+L179*5)</f>
         <v/>
       </c>
       <c r="O179" s="18" t="s"/>
@@ -6436,7 +6436,7 @@
       <c r="L180" s="14" t="s"/>
       <c r="M180" s="14" t="s"/>
       <c r="N180" s="14" t="str">
-        <f>=IF(L180="","",20+L180*5)</f>
+        <f>IF(L180="","",20+L180*5)</f>
         <v/>
       </c>
       <c r="O180" s="18" t="s"/>
@@ -6464,7 +6464,7 @@
       <c r="L181" s="14" t="s"/>
       <c r="M181" s="14" t="s"/>
       <c r="N181" s="14" t="str">
-        <f>=IF(L181="","",20+L181*5)</f>
+        <f>IF(L181="","",20+L181*5)</f>
         <v/>
       </c>
       <c r="O181" s="18" t="s"/>
@@ -6492,7 +6492,7 @@
       <c r="L182" s="14" t="s"/>
       <c r="M182" s="14" t="s"/>
       <c r="N182" s="14" t="str">
-        <f>=IF(L182="","",20+L182*5)</f>
+        <f>IF(L182="","",20+L182*5)</f>
         <v/>
       </c>
       <c r="O182" s="18" t="s"/>
@@ -6520,7 +6520,7 @@
       <c r="L183" s="14" t="s"/>
       <c r="M183" s="14" t="s"/>
       <c r="N183" s="14" t="str">
-        <f>=IF(L183="","",20+L183*5)</f>
+        <f>IF(L183="","",20+L183*5)</f>
         <v/>
       </c>
       <c r="O183" s="18" t="s"/>
@@ -6548,7 +6548,7 @@
       <c r="L184" s="14" t="s"/>
       <c r="M184" s="14" t="s"/>
       <c r="N184" s="14" t="str">
-        <f>=IF(L184="","",20+L184*5)</f>
+        <f>IF(L184="","",20+L184*5)</f>
         <v/>
       </c>
       <c r="O184" s="18" t="s"/>
@@ -6576,7 +6576,7 @@
       <c r="L185" s="14" t="s"/>
       <c r="M185" s="14" t="s"/>
       <c r="N185" s="14" t="str">
-        <f>=IF(L185="","",20+L185*5)</f>
+        <f>IF(L185="","",20+L185*5)</f>
         <v/>
       </c>
       <c r="O185" s="18" t="s"/>
@@ -6604,7 +6604,7 @@
       <c r="L186" s="14" t="s"/>
       <c r="M186" s="14" t="s"/>
       <c r="N186" s="14" t="str">
-        <f>=IF(L186="","",20+L186*5)</f>
+        <f>IF(L186="","",20+L186*5)</f>
         <v/>
       </c>
       <c r="O186" s="18" t="s"/>
@@ -6632,7 +6632,7 @@
       <c r="L187" s="14" t="s"/>
       <c r="M187" s="14" t="s"/>
       <c r="N187" s="14" t="str">
-        <f>=IF(L187="","",20+L187*5)</f>
+        <f>IF(L187="","",20+L187*5)</f>
         <v/>
       </c>
       <c r="O187" s="18" t="s"/>
@@ -6660,7 +6660,7 @@
       <c r="L188" s="14" t="s"/>
       <c r="M188" s="14" t="s"/>
       <c r="N188" s="14" t="str">
-        <f>=IF(L188="","",20+L188*5)</f>
+        <f>IF(L188="","",20+L188*5)</f>
         <v/>
       </c>
       <c r="O188" s="18" t="s"/>
@@ -6688,7 +6688,7 @@
       <c r="L189" s="14" t="s"/>
       <c r="M189" s="14" t="s"/>
       <c r="N189" s="14" t="str">
-        <f>=IF(L189="","",20+L189*5)</f>
+        <f>IF(L189="","",20+L189*5)</f>
         <v/>
       </c>
       <c r="O189" s="18" t="s"/>
@@ -6716,7 +6716,7 @@
       <c r="L190" s="14" t="s"/>
       <c r="M190" s="14" t="s"/>
       <c r="N190" s="14" t="str">
-        <f>=IF(L190="","",20+L190*5)</f>
+        <f>IF(L190="","",20+L190*5)</f>
         <v/>
       </c>
       <c r="O190" s="18" t="s"/>
@@ -6744,7 +6744,7 @@
       <c r="L191" s="14" t="s"/>
       <c r="M191" s="14" t="s"/>
       <c r="N191" s="14" t="str">
-        <f>=IF(L191="","",20+L191*5)</f>
+        <f>IF(L191="","",20+L191*5)</f>
         <v/>
       </c>
       <c r="O191" s="18" t="s"/>
@@ -6772,7 +6772,7 @@
       <c r="L192" s="14" t="s"/>
       <c r="M192" s="14" t="s"/>
       <c r="N192" s="14" t="str">
-        <f>=IF(L192="","",20+L192*5)</f>
+        <f>IF(L192="","",20+L192*5)</f>
         <v/>
       </c>
       <c r="O192" s="18" t="s"/>
@@ -6800,7 +6800,7 @@
       <c r="L193" s="14" t="s"/>
       <c r="M193" s="14" t="s"/>
       <c r="N193" s="14" t="str">
-        <f>=IF(L193="","",20+L193*5)</f>
+        <f>IF(L193="","",20+L193*5)</f>
         <v/>
       </c>
       <c r="O193" s="18" t="s"/>
@@ -6828,7 +6828,7 @@
       <c r="L194" s="14" t="s"/>
       <c r="M194" s="14" t="s"/>
       <c r="N194" s="14" t="str">
-        <f>=IF(L194="","",20+L194*5)</f>
+        <f>IF(L194="","",20+L194*5)</f>
         <v/>
       </c>
       <c r="O194" s="18" t="s"/>
@@ -6856,7 +6856,7 @@
       <c r="L195" s="14" t="s"/>
       <c r="M195" s="14" t="s"/>
       <c r="N195" s="14" t="str">
-        <f>=IF(L195="","",20+L195*5)</f>
+        <f>IF(L195="","",20+L195*5)</f>
         <v/>
       </c>
       <c r="O195" s="18" t="s"/>
@@ -6884,7 +6884,7 @@
       <c r="L196" s="14" t="s"/>
       <c r="M196" s="14" t="s"/>
       <c r="N196" s="14" t="str">
-        <f>=IF(L196="","",20+L196*5)</f>
+        <f>IF(L196="","",20+L196*5)</f>
         <v/>
       </c>
       <c r="O196" s="18" t="s"/>
@@ -6912,7 +6912,7 @@
       <c r="L197" s="14" t="s"/>
       <c r="M197" s="14" t="s"/>
       <c r="N197" s="14" t="str">
-        <f>=IF(L197="","",20+L197*5)</f>
+        <f>IF(L197="","",20+L197*5)</f>
         <v/>
       </c>
       <c r="O197" s="18" t="s"/>
@@ -6940,7 +6940,7 @@
       <c r="L198" s="14" t="s"/>
       <c r="M198" s="14" t="s"/>
       <c r="N198" s="14" t="str">
-        <f>=IF(L198="","",20+L198*5)</f>
+        <f>IF(L198="","",20+L198*5)</f>
         <v/>
       </c>
       <c r="O198" s="18" t="s"/>
@@ -6968,7 +6968,7 @@
       <c r="L199" s="14" t="s"/>
       <c r="M199" s="14" t="s"/>
       <c r="N199" s="14" t="str">
-        <f>=IF(L199="","",20+L199*5)</f>
+        <f>IF(L199="","",20+L199*5)</f>
         <v/>
       </c>
       <c r="O199" s="18" t="s"/>
@@ -6996,7 +6996,7 @@
       <c r="L200" s="14" t="s"/>
       <c r="M200" s="14" t="s"/>
       <c r="N200" s="14" t="str">
-        <f>=IF(L200="","",20+L200*5)</f>
+        <f>IF(L200="","",20+L200*5)</f>
         <v/>
       </c>
       <c r="O200" s="18" t="s"/>
@@ -7024,7 +7024,7 @@
       <c r="L201" s="14" t="s"/>
       <c r="M201" s="14" t="s"/>
       <c r="N201" s="14" t="str">
-        <f>=IF(L201="","",20+L201*5)</f>
+        <f>IF(L201="","",20+L201*5)</f>
         <v/>
       </c>
       <c r="O201" s="18" t="s"/>
@@ -7052,7 +7052,7 @@
       <c r="L202" s="14" t="s"/>
       <c r="M202" s="14" t="s"/>
       <c r="N202" s="14" t="str">
-        <f>=IF(L202="","",20+L202*5)</f>
+        <f>IF(L202="","",20+L202*5)</f>
         <v/>
       </c>
       <c r="O202" s="18" t="s"/>
@@ -7080,7 +7080,7 @@
       <c r="L203" s="14" t="s"/>
       <c r="M203" s="14" t="s"/>
       <c r="N203" s="14" t="str">
-        <f>=IF(L203="","",20+L203*5)</f>
+        <f>IF(L203="","",20+L203*5)</f>
         <v/>
       </c>
       <c r="O203" s="18" t="s"/>

</xml_diff>

<commit_message>
Sync latest design docs and replace chibi art with directional frames
</commit_message>
<xml_diff>
--- a/Excel/Character.xlsx
+++ b/Excel/Character.xlsx
@@ -17,12 +17,12 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>tc={FD08BDE2-6860-4554-85F0-37C9557D8847}</author>
-    <author>tc={6AF71D39-9D17-4F76-BBA8-3E2BDA78960F}</author>
-    <author>tc={616F167E-51F2-446C-978C-FCDCFF1D726C}</author>
-    <author>tc={0BFA0AE2-4038-4DAA-8BF8-1C45B4D2922A}</author>
-    <author>tc={02ECE897-F5AD-4A38-9D26-F436A9B034E3}</author>
-    <author>tc={54BF331E-D745-4386-A204-30D70EAD6E77}</author>
+    <author>tc={72D036DE-F48D-402E-938E-30BA6E2E1FC2}</author>
+    <author>tc={EFB81462-A574-478D-89E4-4B212C90C90C}</author>
+    <author>tc={F2816947-C56A-4550-8A6B-5D7C39F99F2F}</author>
+    <author>tc={FC41775E-F9C5-4B3A-BBFA-D2797082C01B}</author>
+    <author>tc={C8DE027F-7000-412C-A474-B4CADAB99E11}</author>
+    <author>tc={2D9B2A0C-E7FF-4320-9E07-AD9FCEF021EB}</author>
   </authors>
   <commentList>
     <comment ref="E1" authorId="0">
@@ -749,7 +749,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <tc2018:personList xmlns:tc2018="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="tc2018">
-  <tc2018:person displayName="空羽灵" id="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}"/>
+  <tc2018:person displayName="空羽灵" id="{612E3BB4-871E-4BBF-93E0-1299C171BFA7}"/>
 </tc2018:personList>
 </file>
 
@@ -1016,7 +1016,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="">
-  <threadedComment ref="E1" dT="2026-10-08T14:09:11Z" personId="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}" id="{FD08BDE2-6860-4554-85F0-37C9557D8847}">
+  <threadedComment ref="E1" dT="2026-10-08T14:09:11Z" personId="{612E3BB4-871E-4BBF-93E0-1299C171BFA7}" id="{72D036DE-F48D-402E-938E-30BA6E2E1FC2}">
     <text>0=无
 1=厨师
 2=商人
@@ -1026,29 +1026,29 @@
 6=牧师
 7=吟游诗人</text>
   </threadedComment>
-  <threadedComment ref="D1" dT="2026-10-08T14:08:30Z" personId="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}" id="{6AF71D39-9D17-4F76-BBA8-3E2BDA78960F}">
+  <threadedComment ref="D1" dT="2026-10-08T14:08:30Z" personId="{612E3BB4-871E-4BBF-93E0-1299C171BFA7}" id="{EFB81462-A574-478D-89E4-4B212C90C90C}">
     <text>1=男
 2=女</text>
   </threadedComment>
-  <threadedComment ref="Q1" dT="2026-10-08T14:10:50Z" personId="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}" id="{616F167E-51F2-446C-978C-FCDCFF1D726C}">
+  <threadedComment ref="Q1" dT="2026-10-08T14:10:50Z" personId="{612E3BB4-871E-4BBF-93E0-1299C171BFA7}" id="{F2816947-C56A-4550-8A6B-5D7C39F99F2F}">
     <text>1=正常
 2=受伤
 3=中毒
 4=昏迷</text>
   </threadedComment>
-  <threadedComment ref="F1" dT="2026-10-08T14:09:40Z" personId="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}" id="{0BFA0AE2-4038-4DAA-8BF8-1C45B4D2922A}">
+  <threadedComment ref="F1" dT="2026-10-08T14:09:40Z" personId="{612E3BB4-871E-4BBF-93E0-1299C171BFA7}" id="{FC41775E-F9C5-4B3A-BBFA-D2797082C01B}">
     <text>1=开朗
 2=沉稳
 3=谨慎</text>
   </threadedComment>
-  <threadedComment ref="G1" dT="2026-10-08T14:10:05Z" personId="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}" id="{02ECE897-F5AD-4A38-9D26-F436A9B034E3}">
+  <threadedComment ref="G1" dT="2026-10-08T14:10:05Z" personId="{612E3BB4-871E-4BBF-93E0-1299C171BFA7}" id="{C8DE027F-7000-412C-A474-B4CADAB99E11}">
     <text>1=烹饪
 2=锻造
 3=交易
 4=采集
 5=医术</text>
   </threadedComment>
-  <threadedComment ref="P1" dT="2026-10-08T14:10:27Z" personId="{D36F7C4F-01F0-499B-A3F5-7D311C38BBF9}" id="{54BF331E-D745-4386-A204-30D70EAD6E77}">
+  <threadedComment ref="P1" dT="2026-10-08T14:10:27Z" personId="{612E3BB4-871E-4BBF-93E0-1299C171BFA7}" id="{2D9B2A0C-E7FF-4320-9E07-AD9FCEF021EB}">
     <text>1=平静
 2=愉快
 3=低落

</xml_diff>